<commit_message>
Did analysis of all files
</commit_message>
<xml_diff>
--- a/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 26.xlsx
+++ b/BioSensorAnalysisSrcCode/EIS_Analysis/Austin_EIS/MegaExcel/Processed Chips for PCAI1ia/Chip 26.xlsx
@@ -558,8 +558,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>192.894</v>
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-192.894</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.90149e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-82.578</v>
       </c>
       <c r="F2" t="n">
         <v>0.1041068919463167</v>
@@ -584,7 +593,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.156x + -10528.520</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -601,8 +610,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>167.724</v>
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-167.724</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.8692e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-83.01300000000001</v>
       </c>
       <c r="F3" t="n">
         <v>0.3194170350105707</v>
@@ -627,7 +645,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.110x + -11894.280</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -644,8 +662,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>156.5880000000001</v>
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-156.5880000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.8499e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.279</v>
       </c>
       <c r="F4" t="n">
         <v>0.4592797322174187</v>
@@ -670,7 +697,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.604x + -11916.574</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -687,8 +714,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>146.3920000000001</v>
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-146.3920000000001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.83647e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.505</v>
       </c>
       <c r="F5" t="n">
         <v>0.4211102207886185</v>
@@ -713,7 +749,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.037x + -11929.575</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -730,8 +766,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>140.352</v>
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-140.352</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.82578e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.648</v>
       </c>
       <c r="F6" t="n">
         <v>0.7438327345209143</v>
@@ -756,7 +801,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.132x + -12825.707</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -773,8 +818,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>137.215</v>
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-137.215</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.81836e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.807</v>
       </c>
       <c r="F7" t="n">
         <v>0.147417332115022</v>
@@ -799,7 +853,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.466x + -11753.455</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -816,8 +870,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>133.602</v>
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-133.602</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.8107e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.911</v>
       </c>
       <c r="F8" t="n">
         <v>0.5572059038139808</v>
@@ -842,7 +905,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.280x + -12489.765</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -859,8 +922,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>131.738</v>
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-131.738</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.80569e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.02</v>
       </c>
       <c r="F9" t="n">
         <v>0.4414859778278686</v>
@@ -885,7 +957,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.426x + -11877.666</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -902,8 +974,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>128.581</v>
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-128.581</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.80002e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.11499999999999</v>
       </c>
       <c r="F10" t="n">
         <v>0.3162438204802794</v>
@@ -928,7 +1009,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.416x + -12204.342</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -945,8 +1026,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>124.093</v>
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-124.093</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.79627e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.221</v>
       </c>
       <c r="F11" t="n">
         <v>0.4522738789671745</v>
@@ -971,7 +1061,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.049x + -12358.873</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -1134,8 +1224,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>152.723</v>
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-152.723</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.93127e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-83.024</v>
       </c>
       <c r="F2" t="n">
         <v>0.2512352603199477</v>
@@ -1160,7 +1259,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.102x + -10893.998</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -1177,8 +1276,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>131.984</v>
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-131.984</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.92917e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-83.54600000000001</v>
       </c>
       <c r="F3" t="n">
         <v>0.2541025803483765</v>
@@ -1203,7 +1311,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.632x + -11504.339</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -1220,8 +1328,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>129.28</v>
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-129.28</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.9212e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.687</v>
       </c>
       <c r="F4" t="n">
         <v>0.1400792209286618</v>
@@ -1246,7 +1363,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.953x + -11430.260</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -1263,8 +1380,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>124.1009999999999</v>
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-124.1009999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.91187e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.82899999999999</v>
       </c>
       <c r="F5" t="n">
         <v>0.09920623244385056</v>
@@ -1289,7 +1415,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.858x + -11224.706</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -1306,8 +1432,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>119.293</v>
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-119.293</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.90558e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.934</v>
       </c>
       <c r="F6" t="n">
         <v>0.3692688177840676</v>
@@ -1332,7 +1467,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.133x + -12214.074</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -1349,8 +1484,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>117.867</v>
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-117.867</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.90046e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-84.021</v>
       </c>
       <c r="F7" t="n">
         <v>0.2876184136939834</v>
@@ -1375,7 +1519,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.627x + -11820.217</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -1392,8 +1536,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>116.985</v>
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-116.985</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.89592e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-84.09099999999999</v>
       </c>
       <c r="F8" t="n">
         <v>0.3206527290458294</v>
@@ -1418,7 +1571,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.062x + -11887.292</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -1435,8 +1588,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>113.1130000000001</v>
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-113.1130000000001</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.89145e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.19</v>
       </c>
       <c r="F9" t="n">
         <v>0.2387408756064689</v>
@@ -1461,7 +1623,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.648x + -12030.072</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -1478,8 +1640,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>113.2769999999999</v>
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-113.2769999999999</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.88963e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.23</v>
       </c>
       <c r="F10" t="n">
         <v>0.55146302771261</v>
@@ -1504,7 +1675,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.618x + -12366.105</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -1521,8 +1692,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>110.489</v>
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-110.489</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.88777e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.30500000000001</v>
       </c>
       <c r="F11" t="n">
         <v>0.6038148698054053</v>
@@ -1547,7 +1727,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.345x + -12585.917</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -1564,8 +1744,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="n">
-        <v>111.1540000000001</v>
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-111.1540000000001</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.88503e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-84.361</v>
       </c>
       <c r="F12" t="n">
         <v>0.4339865350767734</v>
@@ -1590,7 +1779,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.522x + -12076.695</t>
         </is>
       </c>
       <c r="Y12" t="n">
@@ -1607,8 +1796,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="n">
-        <v>110.27</v>
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-110.27</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.88355e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-84.414</v>
       </c>
       <c r="F13" t="n">
         <v>0.3476471371410548</v>
@@ -1633,7 +1831,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.482x + -11945.455</t>
         </is>
       </c>
       <c r="Y13" t="n">
@@ -1650,8 +1848,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="n">
-        <v>107.432</v>
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-107.432</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.88254e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-84.48099999999999</v>
       </c>
       <c r="F14" t="n">
         <v>0.2703678246490247</v>
@@ -1676,7 +1883,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.217x + -12168.587</t>
         </is>
       </c>
       <c r="Y14" t="n">
@@ -1693,8 +1900,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="n">
-        <v>106.785</v>
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-106.785</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.88131e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-84.52500000000001</v>
       </c>
       <c r="F15" t="n">
         <v>0.3628685771184439</v>
@@ -1719,7 +1935,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.633x + -12247.848</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -1736,8 +1952,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="n">
-        <v>106.9449999999999</v>
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-106.9449999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.87906e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-84.575</v>
       </c>
       <c r="F16" t="n">
         <v>0.3038978515465716</v>
@@ -1762,7 +1987,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.709x + -11721.623</t>
         </is>
       </c>
       <c r="Y16" t="n">
@@ -1779,8 +2004,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="n">
-        <v>112.684</v>
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-112.684</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.87923e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-84.623</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1805,7 +2039,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.129x + -8707.147</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -1822,8 +2056,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="n">
-        <v>102.746</v>
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-102.746</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.87619e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-84.688</v>
       </c>
       <c r="F18" t="n">
         <v>0.4190339336780965</v>
@@ -1848,7 +2091,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.935x + -12491.809</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -1865,8 +2108,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="n">
-        <v>103.851</v>
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-103.851</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.87722e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-84.718</v>
       </c>
       <c r="F19" t="n">
         <v>0.2802140777179493</v>
@@ -1891,7 +2143,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.351x + -12118.932</t>
         </is>
       </c>
       <c r="Y19" t="n">
@@ -1908,8 +2160,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="n">
-        <v>103.498</v>
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-103.498</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.87617e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-84.75700000000001</v>
       </c>
       <c r="F20" t="n">
         <v>0.4864753798457531</v>
@@ -1934,7 +2195,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 30.174x + -12363.801</t>
         </is>
       </c>
       <c r="Y20" t="n">
@@ -1951,8 +2212,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="n">
-        <v>103.721</v>
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-103.721</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.87411e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-84.804</v>
       </c>
       <c r="F21" t="n">
         <v>0.04589902996738593</v>
@@ -1977,7 +2247,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.263x + -11432.831</t>
         </is>
       </c>
       <c r="Y21" t="n">
@@ -1994,8 +2264,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="n">
-        <v>98.95100000000002</v>
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-98.95100000000002</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.87422e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-84.884</v>
       </c>
       <c r="F22" t="n">
         <v>0.4027869637479747</v>
@@ -2020,7 +2299,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 30.629x + -12330.557</t>
         </is>
       </c>
       <c r="Y22" t="n">
@@ -2183,8 +2462,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>185.812</v>
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-185.812</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.86232e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-82.75</v>
       </c>
       <c r="F2" t="n">
         <v>0.3600212400616191</v>
@@ -2209,7 +2497,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.211x + -10616.009</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -2226,8 +2514,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>135.001</v>
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-135.001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.8313e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-83.64400000000001</v>
       </c>
       <c r="F3" t="n">
         <v>0.22385227896093</v>
@@ -2252,7 +2549,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.443x + -12113.065</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -2269,8 +2566,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>126.095</v>
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-126.095</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.82244e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.857</v>
       </c>
       <c r="F4" t="n">
         <v>0.1607162132968337</v>
@@ -2295,7 +2601,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.189x + -11731.888</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -2312,8 +2618,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>117.0359999999999</v>
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-117.0359999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.81385e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-84.01300000000001</v>
       </c>
       <c r="F5" t="n">
         <v>0.4422891215339908</v>
@@ -2338,7 +2653,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.370x + -12691.811</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -2355,8 +2670,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>114.115</v>
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-114.115</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.80933e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-84.089</v>
       </c>
       <c r="F6" t="n">
         <v>0.6625664374199612</v>
@@ -2381,7 +2705,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.434x + -13581.757</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -2398,8 +2722,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>111.591</v>
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-111.591</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.8037e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-84.2</v>
       </c>
       <c r="F7" t="n">
         <v>0.5742009206833052</v>
@@ -2424,7 +2757,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.086x + -12742.011</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -2441,8 +2774,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>113.765</v>
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-113.765</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.79929e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-84.248</v>
       </c>
       <c r="F8" t="n">
         <v>0.2922844361609989</v>
@@ -2467,7 +2809,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.539x + -12321.753</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -2484,8 +2826,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>111.04</v>
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-111.04</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.79486e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.34</v>
       </c>
       <c r="F9" t="n">
         <v>0.2565641828460719</v>
@@ -2510,7 +2861,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.159x + -11994.225</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -2527,8 +2878,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>108.559</v>
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-108.559</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.79076e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.395</v>
       </c>
       <c r="F10" t="n">
         <v>0.5643059452032864</v>
@@ -2553,7 +2913,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.897x + -13193.131</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -2570,8 +2930,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>108.541</v>
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-108.541</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.78869e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.46299999999999</v>
       </c>
       <c r="F11" t="n">
         <v>0.1837260412898271</v>
@@ -2596,7 +2965,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.677x + -11998.704</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -2613,8 +2982,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="n">
-        <v>106.826</v>
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-106.826</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.78439e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-84.51300000000001</v>
       </c>
       <c r="F12" t="n">
         <v>0.5118563139027209</v>
@@ -2639,7 +3017,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.372x + -12691.912</t>
         </is>
       </c>
       <c r="Y12" t="n">
@@ -2656,8 +3034,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="n">
-        <v>104.324</v>
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-104.324</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.78444e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-84.59099999999999</v>
       </c>
       <c r="F13" t="n">
         <v>0.229574198938836</v>
@@ -2682,7 +3069,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.118x + -11990.528</t>
         </is>
       </c>
       <c r="Y13" t="n">
@@ -2699,8 +3086,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="n">
-        <v>102.521</v>
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-102.521</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.78023e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-84.634</v>
       </c>
       <c r="F14" t="n">
         <v>0.434347803510383</v>
@@ -2725,7 +3121,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.840x + -13156.683</t>
         </is>
       </c>
       <c r="Y14" t="n">
@@ -2742,8 +3138,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="n">
-        <v>102.628</v>
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-102.628</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.77878e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-84.67400000000001</v>
       </c>
       <c r="F15" t="n">
         <v>0.3581469239357987</v>
@@ -2768,7 +3173,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.519x + -12896.858</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -2785,8 +3190,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="n">
-        <v>99.24499999999995</v>
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-99.24499999999995</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.77814e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-84.73399999999999</v>
       </c>
       <c r="F16" t="n">
         <v>0.552221576868164</v>
@@ -2811,7 +3225,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 30.535x + -13256.571</t>
         </is>
       </c>
       <c r="Y16" t="n">
@@ -2828,8 +3242,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="n">
-        <v>100.254</v>
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-100.254</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.77535e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-84.78400000000001</v>
       </c>
       <c r="F17" t="n">
         <v>0.05290098768978027</v>
@@ -2854,7 +3277,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.088x + -12033.088</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -2871,8 +3294,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="n">
-        <v>103.455</v>
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-103.455</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.77327e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-84.78700000000001</v>
       </c>
       <c r="F18" t="n">
         <v>0.3624428162188722</v>
@@ -2897,7 +3329,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.585x + -12606.354</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -2914,8 +3346,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="n">
-        <v>101.533</v>
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-101.533</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.77195e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-84.83799999999999</v>
       </c>
       <c r="F19" t="n">
         <v>0.4034514158358037</v>
@@ -2940,7 +3381,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.926x + -12652.627</t>
         </is>
       </c>
       <c r="Y19" t="n">
@@ -2957,8 +3398,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="n">
-        <v>99.31200000000001</v>
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-99.31200000000001</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.77176e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-84.887</v>
       </c>
       <c r="F20" t="n">
         <v>0.6268528781091085</v>
@@ -2983,7 +3433,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 31.396x + -13197.963</t>
         </is>
       </c>
       <c r="Y20" t="n">
@@ -3000,8 +3450,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="n">
-        <v>99.928</v>
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-99.928</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.77071e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-84.929</v>
       </c>
       <c r="F21" t="n">
         <v>0.3365109060421372</v>
@@ -3026,7 +3485,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 29.963x + -12456.513</t>
         </is>
       </c>
       <c r="Y21" t="n">
@@ -3043,8 +3502,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="n">
-        <v>97.21699999999998</v>
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-97.21699999999998</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.76954e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-84.98399999999999</v>
       </c>
       <c r="F22" t="n">
         <v>0.4727542272050645</v>
@@ -3069,7 +3537,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 31.109x + -12847.917</t>
         </is>
       </c>
       <c r="Y22" t="n">
@@ -3232,8 +3700,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>380.9300000000001</v>
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-380.9300000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.18192e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-79.95399999999999</v>
       </c>
       <c r="F2" t="n">
         <v>0.2486354225527059</v>
@@ -3258,7 +3735,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 11.399x + -5628.870</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -3275,8 +3752,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>280.449</v>
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-280.449</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.16511e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-81.804</v>
       </c>
       <c r="F3" t="n">
         <v>0.3106808278072673</v>
@@ -3301,7 +3787,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 15.315x + -6739.300</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -3318,8 +3804,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>238.361</v>
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-238.361</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.11561e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-82.575</v>
       </c>
       <c r="F4" t="n">
         <v>0.03977054612979009</v>
@@ -3344,7 +3839,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 17.593x + -7506.888</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -3361,8 +3856,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>215.98</v>
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-215.98</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.0739e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.045</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -3387,7 +3891,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 18.122x + -7557.433</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -3404,8 +3908,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>192.5579999999999</v>
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-192.5579999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.04238e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.39100000000001</v>
       </c>
       <c r="F6" t="n">
         <v>0.4033259512610427</v>
@@ -3430,7 +3943,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.410x + -8910.350</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -3447,8 +3960,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>180.6729999999999</v>
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-180.6729999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.0168e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.64</v>
       </c>
       <c r="F7" t="n">
         <v>0.4485339825041705</v>
@@ -3473,7 +3995,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.443x + -9214.317</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -3490,8 +4012,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>171.162</v>
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-171.162</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.99736e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.855</v>
       </c>
       <c r="F8" t="n">
         <v>0.2243178878806035</v>
@@ -3516,7 +4047,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.207x + -9385.325</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -3533,8 +4064,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>162.43</v>
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-162.43</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.98304e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.03400000000001</v>
       </c>
       <c r="F9" t="n">
         <v>0.4282541859250891</v>
@@ -3559,7 +4099,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.412x + -9752.118</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -3576,8 +4116,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>162.006</v>
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-162.006</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.96941e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.175</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -3602,7 +4151,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.041x + -8582.619</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -3619,8 +4168,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>149.661</v>
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-149.661</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.95913e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.34399999999999</v>
       </c>
       <c r="F11" t="n">
         <v>0.1837973103988853</v>
@@ -3645,7 +4203,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.189x + -9770.345</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -3808,8 +4366,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>302.482</v>
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-302.482</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.13678e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-80.658</v>
       </c>
       <c r="F2" t="n">
         <v>0.2058765328604114</v>
@@ -3834,7 +4401,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 14.019x + -7342.529</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -3851,8 +4418,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>193.322</v>
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-193.322</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.01041e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-82.495</v>
       </c>
       <c r="F3" t="n">
         <v>0.4803181678963104</v>
@@ -3877,7 +4453,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.640x + -10390.833</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -3894,8 +4470,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>162.029</v>
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-162.029</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.9619e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.06100000000001</v>
       </c>
       <c r="F4" t="n">
         <v>0.3843534950201712</v>
@@ -3920,7 +4505,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.539x + -11150.890</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -3937,8 +4522,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>149.549</v>
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-149.549</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.93403e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.325</v>
       </c>
       <c r="F5" t="n">
         <v>0.2083235471319146</v>
@@ -3963,7 +4557,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.221x + -11336.898</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -3980,8 +4574,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>137.68</v>
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-137.68</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.91834e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.526</v>
       </c>
       <c r="F6" t="n">
         <v>0.6785141872503018</v>
@@ -4006,7 +4609,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.442x + -12337.346</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -4023,8 +4626,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>132.2180000000001</v>
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-132.2180000000001</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.90634e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.682</v>
       </c>
       <c r="F7" t="n">
         <v>0.409746399120797</v>
@@ -4049,7 +4661,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.045x + -11976.821</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -4066,8 +4678,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>126.747</v>
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-126.747</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.89732e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.821</v>
       </c>
       <c r="F8" t="n">
         <v>0.3081169508986153</v>
@@ -4092,7 +4713,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.855x + -11729.212</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -4109,8 +4730,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>126.2839999999999</v>
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-126.2839999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.89073e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-83.89700000000001</v>
       </c>
       <c r="F9" t="n">
         <v>0.3630077700262435</v>
@@ -4135,7 +4765,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.341x + -11836.717</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -4152,8 +4782,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>123.458</v>
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-123.458</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.88377e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.008</v>
       </c>
       <c r="F10" t="n">
         <v>0.0006176672374678497</v>
@@ -4178,7 +4817,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.219x + -11153.355</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -4195,8 +4834,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>119.3849999999999</v>
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-119.3849999999999</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.87984e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.084</v>
       </c>
       <c r="F11" t="n">
         <v>0.1770090710500854</v>
@@ -4221,7 +4869,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.858x + -11838.617</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -4238,8 +4886,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="n">
-        <v>114.622</v>
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-114.622</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.87379e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-84.184</v>
       </c>
       <c r="F12" t="n">
         <v>0.2567083334348363</v>
@@ -4264,7 +4921,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.629x + -12099.651</t>
         </is>
       </c>
       <c r="Y12" t="n">
@@ -4281,8 +4938,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="n">
-        <v>115.45</v>
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-115.45</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.87175e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-84.221</v>
       </c>
       <c r="F13" t="n">
         <v>0.3974558107605298</v>
@@ -4307,7 +4973,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.811x + -12075.262</t>
         </is>
       </c>
       <c r="Y13" t="n">
@@ -4324,8 +4990,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="n">
-        <v>112.47</v>
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-112.47</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.86733e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-84.307</v>
       </c>
       <c r="F14" t="n">
         <v>0.387778184348667</v>
@@ -4350,7 +5025,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.666x + -11892.427</t>
         </is>
       </c>
       <c r="Y14" t="n">
@@ -4367,8 +5042,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="n">
-        <v>111.931</v>
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-111.931</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.86526e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-84.364</v>
       </c>
       <c r="F15" t="n">
         <v>0.07897212754286122</v>
@@ -4393,7 +5077,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.820x + -11390.898</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -4410,8 +5094,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="n">
-        <v>109.052</v>
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-109.052</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.8616e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-84.419</v>
       </c>
       <c r="F16" t="n">
         <v>0.3183689671825659</v>
@@ -4436,7 +5129,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.880x + -12253.841</t>
         </is>
       </c>
       <c r="Y16" t="n">
@@ -4453,8 +5146,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="n">
-        <v>108.99</v>
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-108.99</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.85864e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-84.467</v>
       </c>
       <c r="F17" t="n">
         <v>0.4281340566556781</v>
@@ -4479,7 +5181,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.907x + -12158.414</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -4496,8 +5198,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="n">
-        <v>110.14</v>
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-110.14</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.85582e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-84.497</v>
       </c>
       <c r="F18" t="n">
         <v>0.2587208054347807</v>
@@ -4522,7 +5233,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.725x + -11970.203</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -4539,8 +5250,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="n">
-        <v>104.009</v>
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-104.009</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.85464e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-84.607</v>
       </c>
       <c r="F19" t="n">
         <v>0.2543339516804881</v>
@@ -4565,7 +5285,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.939x + -11512.475</t>
         </is>
       </c>
       <c r="Y19" t="n">
@@ -4582,8 +5302,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="n">
-        <v>106.473</v>
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-106.473</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.85318e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-84.62</v>
       </c>
       <c r="F20" t="n">
         <v>0.3387417122810814</v>
@@ -4608,7 +5337,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.444x + -11638.896</t>
         </is>
       </c>
       <c r="Y20" t="n">
@@ -4625,8 +5354,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="n">
-        <v>103.8749999999999</v>
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-103.8749999999999</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.85219e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-84.67700000000001</v>
       </c>
       <c r="F21" t="n">
         <v>0.2420241148803841</v>
@@ -4651,7 +5389,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.441x + -11981.094</t>
         </is>
       </c>
       <c r="Y21" t="n">
@@ -4668,8 +5406,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="n">
-        <v>101.895</v>
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-101.895</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.85043e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-84.724</v>
       </c>
       <c r="F22" t="n">
         <v>0.3958316044425483</v>
@@ -4694,7 +5441,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 30.299x + -12706.022</t>
         </is>
       </c>
       <c r="Y22" t="n">
@@ -4857,8 +5604,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>415.287</v>
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-415.287</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.33264e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-79.247</v>
       </c>
       <c r="F2" t="n">
         <v>0.1510618611807043</v>
@@ -4883,7 +5639,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 10.022x + -4753.425</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -4900,8 +5656,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>300.403</v>
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-300.403</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.29263e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-81.348</v>
       </c>
       <c r="F3" t="n">
         <v>0.2952116980141143</v>
@@ -4926,7 +5691,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 14.004x + -6004.551</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -4943,8 +5708,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>254.292</v>
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-254.292</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.22555e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-82.224</v>
       </c>
       <c r="F4" t="n">
         <v>0.3234001837650405</v>
@@ -4969,7 +5743,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 16.384x + -6831.824</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -4986,8 +5760,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>223.92</v>
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-223.92</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.17461e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-82.798</v>
       </c>
       <c r="F5" t="n">
         <v>0.2374391016058989</v>
@@ -5012,7 +5795,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 18.175x + -7452.966</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -5029,8 +5812,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>203.7020000000001</v>
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-203.7020000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.13556e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.173</v>
       </c>
       <c r="F6" t="n">
         <v>0.3140501217841745</v>
@@ -5055,7 +5847,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.119x + -8163.711</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -5072,8 +5864,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>189.032</v>
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-189.032</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.10572e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.495</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -5098,7 +5899,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.467x + -8138.085</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -5115,8 +5916,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>177.703</v>
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-177.703</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.08217e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.73</v>
       </c>
       <c r="F8" t="n">
         <v>0.1537407469890794</v>
@@ -5141,7 +5951,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.791x + -8556.790</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -5158,8 +5968,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>169.3899999999999</v>
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-169.3899999999999</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.06404e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-83.94</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -5184,7 +6003,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.106x + -8532.472</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -5201,8 +6020,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>163.521</v>
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-163.521</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.04952e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.096</v>
       </c>
       <c r="F10" t="n">
         <v>0.03565944642924405</v>
@@ -5227,7 +6055,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.508x + -8558.562</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -5244,8 +6072,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>158.2640000000001</v>
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-158.2640000000001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.03864e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.25</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -5270,7 +6107,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.632x + -8073.836</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -5433,8 +6270,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>261.571</v>
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-261.571</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.15126e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-81.19499999999999</v>
       </c>
       <c r="F2" t="n">
         <v>0.4057070833483696</v>
@@ -5459,7 +6305,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 15.482x + -7987.922</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -5476,8 +6322,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>177.236</v>
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-177.236</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.04695e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-82.729</v>
       </c>
       <c r="F3" t="n">
         <v>0.6238346451875197</v>
@@ -5502,7 +6357,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.303x + -10453.379</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -5519,8 +6374,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>157.1960000000001</v>
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-157.1960000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.00868e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.166</v>
       </c>
       <c r="F4" t="n">
         <v>0.06818604703665022</v>
@@ -5545,7 +6409,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.580x + -10342.095</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -5562,8 +6426,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>145.2930000000001</v>
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-145.2930000000001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.98863e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.399</v>
       </c>
       <c r="F5" t="n">
         <v>0.1110759864314674</v>
@@ -5588,7 +6461,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.514x + -10665.842</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -5605,8 +6478,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>136.829</v>
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-136.829</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.97582e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.568</v>
       </c>
       <c r="F6" t="n">
         <v>0.241685382853705</v>
@@ -5631,7 +6513,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.679x + -11109.854</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -5648,8 +6530,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>129.434</v>
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-129.434</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.96574e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.73099999999999</v>
       </c>
       <c r="F7" t="n">
         <v>0.4195948978627454</v>
@@ -5674,7 +6565,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.693x + -11470.745</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -5691,8 +6582,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>129.434</v>
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-129.434</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.95844e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.81999999999999</v>
       </c>
       <c r="F8" t="n">
         <v>0.05522112977547446</v>
@@ -5717,7 +6617,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.829x + -10899.961</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -5734,8 +6634,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>122.062</v>
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-122.062</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.9517e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-83.932</v>
       </c>
       <c r="F9" t="n">
         <v>0.6766973606147526</v>
@@ -5760,7 +6669,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.740x + -12184.708</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -5777,8 +6686,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>121.4230000000001</v>
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-121.4230000000001</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.94842e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.015</v>
       </c>
       <c r="F10" t="n">
         <v>0.1889606284772116</v>
@@ -5803,7 +6721,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.126x + -11277.142</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -5820,8 +6738,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>118.37</v>
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-118.37</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.94245e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.111</v>
       </c>
       <c r="F11" t="n">
         <v>0.4119672874672737</v>
@@ -5846,7 +6773,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.212x + -11202.344</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -5863,8 +6790,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="n">
-        <v>117.152</v>
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-117.152</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.93913e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-84.166</v>
       </c>
       <c r="F12" t="n">
         <v>0.3924705789042351</v>
@@ -5889,7 +6825,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.012x + -11467.553</t>
         </is>
       </c>
       <c r="Y12" t="n">
@@ -5906,8 +6842,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="n">
-        <v>114.402</v>
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-114.402</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.93662e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-84.233</v>
       </c>
       <c r="F13" t="n">
         <v>0.5272546335985324</v>
@@ -5932,7 +6877,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.843x + -11745.343</t>
         </is>
       </c>
       <c r="Y13" t="n">
@@ -5949,8 +6894,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="n">
-        <v>114.677</v>
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-114.677</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.93307e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-84.288</v>
       </c>
       <c r="F14" t="n">
         <v>0.2596611031854913</v>
@@ -5975,7 +6929,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.416x + -11435.601</t>
         </is>
       </c>
       <c r="Y14" t="n">
@@ -5992,8 +6946,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="n">
-        <v>109.143</v>
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-109.143</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.93089e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-84.396</v>
       </c>
       <c r="F15" t="n">
         <v>0.2126113263100747</v>
@@ -6018,7 +6981,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.727x + -11468.043</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -6035,8 +6998,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="n">
-        <v>106.725</v>
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-106.725</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.92741e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-84.45699999999999</v>
       </c>
       <c r="F16" t="n">
         <v>0.3853431843905843</v>
@@ -6061,7 +7033,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.433x + -11676.233</t>
         </is>
       </c>
       <c r="Y16" t="n">
@@ -6078,8 +7050,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="n">
-        <v>108.109</v>
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-108.109</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.92711e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-84.498</v>
       </c>
       <c r="F17" t="n">
         <v>0.3312520345965826</v>
@@ -6104,7 +7085,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.257x + -11042.483</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -6121,8 +7102,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="n">
-        <v>115.366</v>
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-115.366</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.92538e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-84.541</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -6147,7 +7137,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 19.702x + -8057.979</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -6164,8 +7154,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="n">
-        <v>103.657</v>
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-103.657</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.92352e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-84.61499999999999</v>
       </c>
       <c r="F19" t="n">
         <v>0.6011164811750711</v>
@@ -6190,7 +7189,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.465x + -11809.416</t>
         </is>
       </c>
       <c r="Y19" t="n">
@@ -6207,8 +7206,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="n">
-        <v>103.911</v>
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-103.911</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.92278e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-84.658</v>
       </c>
       <c r="F20" t="n">
         <v>0.4060632175973847</v>
@@ -6233,7 +7241,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.233x + -11595.304</t>
         </is>
       </c>
       <c r="Y20" t="n">
@@ -6250,8 +7258,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="n">
-        <v>108.898</v>
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-108.898</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.92051e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-84.7</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -6276,7 +7293,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.049x + -9258.846</t>
         </is>
       </c>
       <c r="Y21" t="n">
@@ -6293,8 +7310,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="n">
-        <v>102.782</v>
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-102.782</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.92126e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-84.748</v>
       </c>
       <c r="F22" t="n">
         <v>0.3460987541429899</v>
@@ -6319,7 +7345,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.659x + -11563.321</t>
         </is>
       </c>
       <c r="Y22" t="n">
@@ -6482,8 +7508,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>393.725</v>
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-393.725</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.35159e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-79.379</v>
       </c>
       <c r="F2" t="n">
         <v>0.3355328595150014</v>
@@ -6508,7 +7543,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 10.542x + -5076.239</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -6525,8 +7560,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>278.3680000000001</v>
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-278.3680000000001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.28991e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-81.65600000000001</v>
       </c>
       <c r="F3" t="n">
         <v>0.1603454460234977</v>
@@ -6551,7 +7595,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 14.678x + -6259.777</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -6568,8 +7612,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>227.635</v>
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-227.635</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.21697e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-82.571</v>
       </c>
       <c r="F4" t="n">
         <v>0.6273173030063035</v>
@@ -6594,7 +7647,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 18.208x + -7592.345</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -6611,8 +7664,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>198.654</v>
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-198.654</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.16364e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.12</v>
       </c>
       <c r="F5" t="n">
         <v>0.4251616491959277</v>
@@ -6637,7 +7699,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 19.918x + -8153.215</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -6654,8 +7716,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>181.672</v>
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-181.672</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.12615e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.468</v>
       </c>
       <c r="F6" t="n">
         <v>0.2104298985136608</v>
@@ -6680,7 +7751,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.281x + -8592.884</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -6697,8 +7768,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>168.712</v>
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-168.712</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3.09917e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.755</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -6723,7 +7803,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.657x + -8593.149</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -6740,8 +7820,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>158.627</v>
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-158.627</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3.07858e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.965</v>
       </c>
       <c r="F8" t="n">
         <v>0.1512018233207274</v>
@@ -6766,7 +7855,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.704x + -8896.116</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -6783,8 +7872,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>152.704</v>
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-152.704</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3.06218e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.107</v>
       </c>
       <c r="F9" t="n">
         <v>0.360155359749003</v>
@@ -6809,7 +7907,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.138x + -9358.576</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -6826,8 +7924,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>145.009</v>
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-145.009</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.05109e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.29000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>0.1289736245424689</v>
@@ -6852,7 +7959,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.381x + -8897.997</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -6869,8 +7976,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>140.537</v>
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-140.537</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3.04068e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.393</v>
       </c>
       <c r="F11" t="n">
         <v>0.2649344826764415</v>
@@ -6895,7 +8011,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.351x + -9576.223</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -7058,8 +8174,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>248.224</v>
+      <c r="A2" t="n">
+        <v>1.428571428571429</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-248.224</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.16062e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-81.358</v>
       </c>
       <c r="F2" t="n">
         <v>0.1533710651901444</v>
@@ -7084,7 +8209,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 15.651x + -8041.755</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -7101,8 +8226,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>174.905</v>
+      <c r="A3" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-174.905</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.06331e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-82.718</v>
       </c>
       <c r="F3" t="n">
         <v>0.167238872282497</v>
@@ -7127,7 +8261,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.238x + -9910.927</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -7144,8 +8278,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>151.73</v>
+      <c r="A4" t="n">
+        <v>4.285714285714286</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-151.73</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.02365e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.161</v>
       </c>
       <c r="F4" t="n">
         <v>0.118683459369862</v>
@@ -7170,7 +8313,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.874x + -10531.451</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -7187,8 +8330,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>140.738</v>
+      <c r="A5" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-140.738</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.00137e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.40600000000001</v>
       </c>
       <c r="F5" t="n">
         <v>0.4456917023317447</v>
@@ -7213,7 +8365,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.873x + -10873.962</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -7230,8 +8382,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>133.039</v>
+      <c r="A6" t="n">
+        <v>7.142857142857143</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-133.039</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.98912e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-83.601</v>
       </c>
       <c r="F6" t="n">
         <v>0.1273861864446729</v>
@@ -7256,7 +8417,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.296x + -10421.739</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -7273,8 +8434,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>127.572</v>
+      <c r="A7" t="n">
+        <v>8.571428571428571</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-127.572</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.97741e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-83.742</v>
       </c>
       <c r="F7" t="n">
         <v>0.05249041822420263</v>
@@ -7299,7 +8469,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.202x + -10718.833</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -7316,8 +8486,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>124.5119999999999</v>
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-124.5119999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.97057e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-83.855</v>
       </c>
       <c r="F8" t="n">
         <v>0.1700647641337131</v>
@@ -7342,7 +8521,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.800x + -10854.508</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -7359,8 +8538,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>118.5140000000001</v>
+      <c r="A9" t="n">
+        <v>11.42857142857143</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-118.5140000000001</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.96572e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-83.97499999999999</v>
       </c>
       <c r="F9" t="n">
         <v>0.5752312257961332</v>
@@ -7385,7 +8573,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.141x + -11833.508</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -7402,8 +8590,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>119.23</v>
+      <c r="A10" t="n">
+        <v>12.85714285714286</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-119.23</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.95921e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.054</v>
       </c>
       <c r="F10" t="n">
         <v>0.2813013731631299</v>
@@ -7428,7 +8625,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.099x + -11191.991</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -7445,8 +8642,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>115.397</v>
+      <c r="A11" t="n">
+        <v>14.28571428571429</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-115.397</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.95583e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.151</v>
       </c>
       <c r="F11" t="n">
         <v>0.09319130765298622</v>
@@ -7471,7 +8677,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.179x + -11088.938</t>
         </is>
       </c>
       <c r="Y11" t="n">
@@ -7488,8 +8694,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="C12" t="n">
-        <v>115.532</v>
+      <c r="A12" t="n">
+        <v>15.71428571428572</v>
+      </c>
+      <c r="B12" t="n">
+        <v>-115.532</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2.95296e-07</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-84.20099999999999</v>
       </c>
       <c r="F12" t="n">
         <v>0.3599413389630866</v>
@@ -7514,7 +8729,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 26.189x + -11435.848</t>
         </is>
       </c>
       <c r="Y12" t="n">
@@ -7531,8 +8746,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="C13" t="n">
-        <v>111.609</v>
+      <c r="A13" t="n">
+        <v>17.14285714285714</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-111.609</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.94949e-07</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-84.303</v>
       </c>
       <c r="F13" t="n">
         <v>0.1708077574308895</v>
@@ -7557,7 +8781,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.829x + -11145.944</t>
         </is>
       </c>
       <c r="Y13" t="n">
@@ -7574,8 +8798,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="C14" t="n">
-        <v>105.909</v>
+      <c r="A14" t="n">
+        <v>18.57142857142857</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-105.909</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.94769e-07</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-84.392</v>
       </c>
       <c r="F14" t="n">
         <v>0.5627007889638423</v>
@@ -7600,7 +8833,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.565x + -11825.718</t>
         </is>
       </c>
       <c r="Y14" t="n">
@@ -7617,8 +8850,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="C15" t="n">
-        <v>109.815</v>
+      <c r="A15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-109.815</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2.94521e-07</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-84.419</v>
       </c>
       <c r="F15" t="n">
         <v>0.2204768402855436</v>
@@ -7643,7 +8885,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 25.916x + -10963.163</t>
         </is>
       </c>
       <c r="Y15" t="n">
@@ -7660,8 +8902,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" t="n">
-        <v>106.6619999999999</v>
+      <c r="A16" t="n">
+        <v>21.42857142857143</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-106.6619999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.94213e-07</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-84.486</v>
       </c>
       <c r="F16" t="n">
         <v>0.4084886904978213</v>
@@ -7686,7 +8937,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.726x + -11663.678</t>
         </is>
       </c>
       <c r="Y16" t="n">
@@ -7703,8 +8954,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="C17" t="n">
-        <v>105.321</v>
+      <c r="A17" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-105.321</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2.94177e-07</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-84.547</v>
       </c>
       <c r="F17" t="n">
         <v>0.3421720146806932</v>
@@ -7729,7 +8989,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.323x + -11367.490</t>
         </is>
       </c>
       <c r="Y17" t="n">
@@ -7746,8 +9006,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="C18" t="n">
-        <v>104.587</v>
+      <c r="A18" t="n">
+        <v>24.28571428571428</v>
+      </c>
+      <c r="B18" t="n">
+        <v>-104.587</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.93998e-07</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-84.598</v>
       </c>
       <c r="F18" t="n">
         <v>0.3530225523922933</v>
@@ -7772,7 +9041,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.356x + -11271.295</t>
         </is>
       </c>
       <c r="Y18" t="n">
@@ -7789,8 +9058,17 @@
       </c>
     </row>
     <row r="19">
-      <c r="C19" t="n">
-        <v>102.743</v>
+      <c r="A19" t="n">
+        <v>25.71428571428572</v>
+      </c>
+      <c r="B19" t="n">
+        <v>-102.743</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.93884e-07</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-84.655</v>
       </c>
       <c r="F19" t="n">
         <v>0.50489475641645</v>
@@ -7815,7 +9093,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.334x + -11585.463</t>
         </is>
       </c>
       <c r="Y19" t="n">
@@ -7832,8 +9110,17 @@
       </c>
     </row>
     <row r="20">
-      <c r="C20" t="n">
-        <v>101.33</v>
+      <c r="A20" t="n">
+        <v>27.14285714285714</v>
+      </c>
+      <c r="B20" t="n">
+        <v>-101.33</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.93564e-07</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-84.729</v>
       </c>
       <c r="F20" t="n">
         <v>0.2225979619249348</v>
@@ -7858,7 +9145,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.440x + -11087.491</t>
         </is>
       </c>
       <c r="Y20" t="n">
@@ -7875,8 +9162,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="C21" t="n">
-        <v>100.533</v>
+      <c r="A21" t="n">
+        <v>28.57142857142857</v>
+      </c>
+      <c r="B21" t="n">
+        <v>-100.533</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2.93534e-07</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-84.773</v>
       </c>
       <c r="F21" t="n">
         <v>0.08864719402297366</v>
@@ -7901,7 +9197,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.784x + -11127.632</t>
         </is>
       </c>
       <c r="Y21" t="n">
@@ -7918,8 +9214,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="C22" t="n">
-        <v>99.27299999999997</v>
+      <c r="A22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-99.27299999999997</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.93414e-07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-84.828</v>
       </c>
       <c r="F22" t="n">
         <v>0.2331695885852351</v>
@@ -7944,7 +9249,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 28.537x + -11332.965</t>
         </is>
       </c>
       <c r="Y22" t="n">
@@ -8107,8 +9412,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" t="n">
-        <v>375.6270000000001</v>
+      <c r="A2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-375.6270000000001</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.22643e-07</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-80.02800000000001</v>
       </c>
       <c r="F2" t="n">
         <v>0.3090341367424562</v>
@@ -8133,7 +9447,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 11.197x + -5404.923</t>
         </is>
       </c>
       <c r="Y2" t="n">
@@ -8150,8 +9464,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" t="n">
-        <v>250.0069999999999</v>
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>-250.0069999999999</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.16105e-07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-82.399</v>
       </c>
       <c r="F3" t="n">
         <v>0.2408363026047992</v>
@@ -8176,7 +9499,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 16.638x + -7005.263</t>
         </is>
       </c>
       <c r="Y3" t="n">
@@ -8193,8 +9516,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" t="n">
-        <v>203.114</v>
+      <c r="A4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B4" t="n">
+        <v>-203.114</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.09133e-07</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-83.236</v>
       </c>
       <c r="F4" t="n">
         <v>0.3624615440235107</v>
@@ -8219,7 +9551,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 20.052x + -8202.643</t>
         </is>
       </c>
       <c r="Y4" t="n">
@@ -8236,8 +9568,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" t="n">
-        <v>178.4640000000001</v>
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>-178.4640000000001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.04231e-07</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-83.7</v>
       </c>
       <c r="F5" t="n">
         <v>0.06844359911676329</v>
@@ -8262,7 +9603,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 21.874x + -8793.680</t>
         </is>
       </c>
       <c r="Y5" t="n">
@@ -8279,8 +9620,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" t="n">
-        <v>157.437</v>
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>-157.437</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3.01126e-07</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-84.06100000000001</v>
       </c>
       <c r="F6" t="n">
         <v>0.1555675523765995</v>
@@ -8305,7 +9655,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.747x + -9406.969</t>
         </is>
       </c>
       <c r="Y6" t="n">
@@ -8322,8 +9672,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" t="n">
-        <v>150.675</v>
+      <c r="A7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B7" t="n">
+        <v>-150.675</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.99036e-07</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-84.277</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -8348,7 +9707,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.481x + -8700.101</t>
         </is>
       </c>
       <c r="Y7" t="n">
@@ -8365,8 +9724,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="C8" t="n">
-        <v>146.104</v>
+      <c r="A8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-146.104</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.97612e-07</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-84.42100000000001</v>
       </c>
       <c r="F8" t="n">
         <v>0.0005794371424074043</v>
@@ -8391,7 +9759,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 22.976x + -8746.054</t>
         </is>
       </c>
       <c r="Y8" t="n">
@@ -8408,8 +9776,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="C9" t="n">
-        <v>137.07</v>
+      <c r="A9" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
+        <v>-137.07</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.9661e-07</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-84.605</v>
       </c>
       <c r="F9" t="n">
         <v>0.03656112523676364</v>
@@ -8434,7 +9811,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 23.548x + -8815.579</t>
         </is>
       </c>
       <c r="Y9" t="n">
@@ -8451,8 +9828,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" t="n">
-        <v>130.099</v>
+      <c r="A10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-130.099</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.95805e-07</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-84.70999999999999</v>
       </c>
       <c r="F10" t="n">
         <v>0.8745145247774707</v>
@@ -8477,7 +9863,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 27.703x + -10328.277</t>
         </is>
       </c>
       <c r="Y10" t="n">
@@ -8494,8 +9880,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" t="n">
-        <v>129.637</v>
+      <c r="A11" t="n">
+        <v>30</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-129.637</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.95183e-07</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-84.83199999999999</v>
       </c>
       <c r="F11" t="n">
         <v>0.0576374564442183</v>
@@ -8520,7 +9915,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>CPE</t>
+          <t>y = 24.131x + -8761.432</t>
         </is>
       </c>
       <c r="Y11" t="n">

</xml_diff>